<commit_message>
Complete private parsing benchmark reproducibility
</commit_message>
<xml_diff>
--- a/document-parsing/evaluate/idc-4.1.14_半导体场景模拟数据_解析benchmark评分.xlsx
+++ b/document-parsing/evaluate/idc-4.1.14_半导体场景模拟数据_解析benchmark评分.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2cba687d3f484781"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scores" sheetId="2" r:id="R0d3c88e8c0f845fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension Details" sheetId="3" r:id="Rabed77404af745cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3f04a04f6b1548b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scores" sheetId="2" r:id="R6638a0dd75564afb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dimension Details" sheetId="3" r:id="Rfd1a0581e78840d2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -122,7 +122,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1"/>
@@ -187,6 +187,9 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -466,11 +469,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
-    <x:col min="1" max="1" width="32" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="13.890000343322754" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="10.329999923706055" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="18.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="9.109999656677246" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -496,7 +499,7 @@
       <x:c r="G2"/>
       <x:c r="H2"/>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3" ht="32" hidden="0" customHeight="1">
       <x:c r="A3" s="15" t="str">
         <x:v>Product</x:v>
       </x:c>
@@ -511,10 +514,10 @@
         <x:v>Contributing files</x:v>
       </x:c>
       <x:c r="F3" s="21" t="str">
-        <x:v>F1 equal avg</x:v>
+        <x:v>Per-dimension F1 avg across files</x:v>
       </x:c>
       <x:c r="G3" s="21" t="str">
-        <x:v>F1 count-weighted avg</x:v>
+        <x:v>Per-dimension F1 weighted by all elements</x:v>
       </x:c>
       <x:c r="H3" s="21" t="str">
         <x:v>Total count</x:v>
@@ -595,24 +598,24 @@
       </x:c>
       <x:c r="F6" s="22" t="n">
         <x:f>AVERAGE('Scores'!H2:H51)</x:f>
-        <x:v>0.8472949999999999</x:v>
+        <x:v>0.797295</x:v>
       </x:c>
       <x:c r="G6" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!H2:H51,'Scores'!R2:R51)/SUM('Scores'!R2:R51)</x:f>
-        <x:v>0.8882846153846155</x:v>
+        <x:v>0.7921307692307693</x:v>
       </x:c>
       <x:c r="H6" s="16" t="n">
         <x:f>SUM('Scores'!R2:R51)</x:f>
         <x:v>52</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="15" t="str">
-        <x:v>Avg equal-weight score across files</x:v>
+    <x:row r="7" ht="30" hidden="0" customHeight="1">
+      <x:c r="A7" s="25" t="str">
+        <x:v>50-file avg of per-file dimension-equal scores</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
         <x:f>AVERAGE('Scores'!Y2:Y51)</x:f>
-        <x:v>0.8492585809523806</x:v>
+        <x:v>0.8445537238095235</x:v>
       </x:c>
       <x:c r="C7"/>
       <x:c r="D7" s="16" t="str">
@@ -624,24 +627,24 @@
       </x:c>
       <x:c r="F7" s="22" t="n">
         <x:f>AVERAGE('Scores'!I2:I51)</x:f>
-        <x:v>0.9664119999999998</x:v>
+        <x:v>0.9640719999999997</x:v>
       </x:c>
       <x:c r="G7" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!I2:I51,'Scores'!S2:S51)/SUM('Scores'!S2:S51)</x:f>
-        <x:v>0.9805639736684622</x:v>
+        <x:v>0.9781833632555358</x:v>
       </x:c>
       <x:c r="H7" s="16" t="n">
         <x:f>SUM('Scores'!S2:S51)</x:f>
         <x:v>1671</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="58" hidden="0" customHeight="1">
-      <x:c r="A8" s="15" t="str">
-        <x:v>Avg count-weighted score across files</x:v>
+    <x:row r="8" ht="30" hidden="0" customHeight="1">
+      <x:c r="A8" s="25" t="str">
+        <x:v>50-file avg of per-file element-count-weighted scores</x:v>
       </x:c>
       <x:c r="B8" s="17" t="n">
         <x:f>AVERAGE('Scores'!Z2:Z51)</x:f>
-        <x:v>0.8962932604828109</x:v>
+        <x:v>0.893841460941976</x:v>
       </x:c>
       <x:c r="C8"/>
       <x:c r="D8" s="16" t="str">
@@ -653,11 +656,11 @@
       </x:c>
       <x:c r="F8" s="22" t="n">
         <x:f>AVERAGE('Scores'!K2:K51)</x:f>
-        <x:v>0.852525641025641</x:v>
+        <x:v>0.8459641025641025</x:v>
       </x:c>
       <x:c r="G8" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!K2:K51,'Scores'!U2:U51)/SUM('Scores'!U2:U51)</x:f>
-        <x:v>0.8557669642857142</x:v>
+        <x:v>0.853474107142857</x:v>
       </x:c>
       <x:c r="H8" s="16" t="n">
         <x:f>SUM('Scores'!U2:U51)</x:f>
@@ -666,10 +669,10 @@
     </x:row>
     <x:row r="9" ht="42" hidden="0" customHeight="1">
       <x:c r="A9" s="15" t="str">
-        <x:v>Evaluation run</x:v>
+        <x:v>Evaluation provenance</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>eval_20260731_034612_dbc092</x:v>
+        <x:v>tracked ZIPs + score_semiconductor_private.py</x:v>
       </x:c>
       <x:c r="C9"/>
       <x:c r="D9" s="16" t="str">
@@ -681,11 +684,11 @@
       </x:c>
       <x:c r="F9" s="22" t="n">
         <x:f>AVERAGE('Scores'!L2:L51)</x:f>
-        <x:v>0.7396743589743588</x:v>
+        <x:v>0.7313179487179488</x:v>
       </x:c>
       <x:c r="G9" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!L2:L51,'Scores'!V2:V51)/SUM('Scores'!V2:V51)</x:f>
-        <x:v>0.7201625</x:v>
+        <x:v>0.7167562500000001</x:v>
       </x:c>
       <x:c r="H9" s="16" t="n">
         <x:f>SUM('Scores'!V2:V51)</x:f>
@@ -709,11 +712,11 @@
       </x:c>
       <x:c r="F10" s="22" t="n">
         <x:f>AVERAGE('Scores'!M2:M51)</x:f>
-        <x:v>0.8253404761904763</x:v>
+        <x:v>0.8265904761904762</x:v>
       </x:c>
       <x:c r="G10" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!M2:M51,'Scores'!W2:W51)/SUM('Scores'!W2:W51)</x:f>
-        <x:v>0.9321093984962407</x:v>
+        <x:v>0.9329862781954888</x:v>
       </x:c>
       <x:c r="H10" s="16" t="n">
         <x:f>SUM('Scores'!W2:W51)</x:f>
@@ -722,10 +725,10 @@
     </x:row>
     <x:row r="11" ht="42" hidden="0" customHeight="1">
       <x:c r="A11" s="15" t="str">
-        <x:v>Golden snapshots</x:v>
+        <x:v>Golden directory</x:v>
       </x:c>
       <x:c r="B11" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens</x:v>
+        <x:v>datasets/半导体场景模拟数据golden</x:v>
       </x:c>
       <x:c r="C11"/>
       <x:c r="D11" s="16" t="str">
@@ -737,11 +740,11 @@
       </x:c>
       <x:c r="F11" s="22" t="n">
         <x:f>AVERAGE('Scores'!N2:N51)</x:f>
-        <x:v>0.8703047619047618</x:v>
+        <x:v>0.8708333333333332</x:v>
       </x:c>
       <x:c r="G11" s="22" t="n">
         <x:f>SUMPRODUCT('Scores'!N2:N51,'Scores'!X2:X51)/SUM('Scores'!X2:X51)</x:f>
-        <x:v>0.9173191873589164</x:v>
+        <x:v>0.9183214446952597</x:v>
       </x:c>
       <x:c r="H11" s="16" t="n">
         <x:f>SUM('Scores'!X2:X51)</x:f>
@@ -784,15 +787,15 @@
     <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
     <x:col min="23" max="23" width="17.670000076293945" hidden="0" customWidth="1"/>
     <x:col min="24" max="24" width="19" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="18.219999313354492" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="20.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="36" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="36" hidden="0" customWidth="1"/>
     <x:col min="27" max="27" width="16.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="28" max="28" width="60" hidden="0" customWidth="1"/>
     <x:col min="29" max="29" width="60" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="60" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="15" hidden="0" customHeight="1">
+    <x:row r="1" ht="32" hidden="0" customHeight="1">
       <x:c r="A1" s="21" t="str">
         <x:v>case_name</x:v>
       </x:c>
@@ -866,10 +869,10 @@
         <x:v>title_hierarchy_count</x:v>
       </x:c>
       <x:c r="Y1" s="21" t="str">
-        <x:v>equal_weight_score</x:v>
+        <x:v>per_file_dimension_equal_score</x:v>
       </x:c>
       <x:c r="Z1" s="21" t="str">
-        <x:v>count_weighted_score</x:v>
+        <x:v>per_file_element_count_weighted_score</x:v>
       </x:c>
       <x:c r="AA1" s="21" t="str">
         <x:v>tool_overall_score</x:v>
@@ -951,13 +954,13 @@
         <x:v>0.9772</x:v>
       </x:c>
       <x:c r="AB2" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/0625-case_d39d394f8a/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/0625跨页表合并复现case.docx--be16ef7e1cbf.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC2" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/0625-case_d39d394f8a.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/0625跨页表合并复现case.docx.json</x:v>
       </x:c>
       <x:c r="AD2" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/0625跨页表合并复现case.docx--be16ef7e1cbf.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -1031,13 +1034,13 @@
         <x:v>0.9097</x:v>
       </x:c>
       <x:c r="AB3" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/08_713a323249/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08标题识别为页眉.pptx--7234c9311c55.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC3" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/08_713a323249.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/08标题识别为页眉.pptx.json</x:v>
       </x:c>
       <x:c r="AD3" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08标题识别为页眉.pptx--7234c9311c55.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1099,13 +1102,13 @@
         <x:v>0.9491</x:v>
       </x:c>
       <x:c r="AB4" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/08_f7c25b83c3/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页眉页脚多识别.pptx--0ded5f710a55.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC4" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/08_f7c25b83c3.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/08页眉页脚多识别.pptx.json</x:v>
       </x:c>
       <x:c r="AD4" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页眉页脚多识别.pptx--0ded5f710a55.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -1171,13 +1174,13 @@
         <x:v>0.9508</x:v>
       </x:c>
       <x:c r="AB5" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/08_389a4aee4c/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页面的标题相似度高被当做页眉.pptx--3907ec0c31cf.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC5" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/08_389a4aee4c.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/08页面的标题相似度高被当做页眉.pptx.json</x:v>
       </x:c>
       <x:c r="AD5" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页面的标题相似度高被当做页眉.pptx--3907ec0c31cf.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -1243,13 +1246,13 @@
         <x:v>0.8536</x:v>
       </x:c>
       <x:c r="AB6" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/112_3881eae9f9/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/112跨页表解析两次.docx--014918d9abd9.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC6" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/112_3881eae9f9.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/112跨页表解析两次.docx.json</x:v>
       </x:c>
       <x:c r="AD6" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/112跨页表解析两次.docx--014918d9abd9.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -1319,13 +1322,13 @@
         <x:v>0.9424</x:v>
       </x:c>
       <x:c r="AB7" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/114-_old_274e089043/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/114跨页表识别为两张表_old.docx--8ec7f5aca322.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC7" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/114-_old_274e089043.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/114跨页表识别为两张表_old.docx.json</x:v>
       </x:c>
       <x:c r="AD7" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/114跨页表识别为两张表_old.docx--8ec7f5aca322.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -1387,13 +1390,13 @@
         <x:v>0.8637</x:v>
       </x:c>
       <x:c r="AB8" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/115_f58f4b08cd/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/115标题在文档中间.pptx--e04aea954be4.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC8" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/115_f58f4b08cd.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/115标题在文档中间.pptx.json</x:v>
       </x:c>
       <x:c r="AD8" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/115标题在文档中间.pptx--e04aea954be4.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -1459,13 +1462,13 @@
         <x:v>0.75</x:v>
       </x:c>
       <x:c r="AB9" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/12-__f685acd93c/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12表格不合并单元格错乱_居中.pptx--7883fda78449.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC9" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/12-__f685acd93c.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/12表格不合并单元格错乱_居中.pptx.json</x:v>
       </x:c>
       <x:c r="AD9" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12表格不合并单元格错乱_居中.pptx--7883fda78449.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -1535,13 +1538,13 @@
         <x:v>0.9576</x:v>
       </x:c>
       <x:c r="AB10" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/12-__fd2ba7ab8d/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12测试跨页表的拼接_每页有表头.docx--6b2bf687f300.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC10" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/12-__fd2ba7ab8d.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/12测试跨页表的拼接_每页有表头.docx.json</x:v>
       </x:c>
       <x:c r="AD10" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12测试跨页表的拼接_每页有表头.docx--6b2bf687f300.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1607,13 +1610,13 @@
         <x:v>0.5702</x:v>
       </x:c>
       <x:c r="AB11" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/12_6ec5e722c7/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12测试跨页表的拼接.pdf--47a16cb613a6.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC11" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/12_6ec5e722c7.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/12测试跨页表的拼接.pdf.json</x:v>
       </x:c>
       <x:c r="AD11" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12测试跨页表的拼接.pdf--47a16cb613a6.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1687,13 +1690,13 @@
         <x:v>0.9169</x:v>
       </x:c>
       <x:c r="AB12" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/12_cae6a0c1bf/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12多线表跨页拼接.pdf--5bd92a999b34.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC12" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/12_cae6a0c1bf.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/12多线表跨页拼接.pdf.json</x:v>
       </x:c>
       <x:c r="AD12" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/12多线表跨页拼接.pdf--5bd92a999b34.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -1767,13 +1770,13 @@
         <x:v>0.957</x:v>
       </x:c>
       <x:c r="AB13" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/145_b2ca7bd18e/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/145页眉下的图片被识别为表格一部分.docx--2aafe56f9445.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC13" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/145_b2ca7bd18e.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/145页眉下的图片被识别为表格一部分.docx.json</x:v>
       </x:c>
       <x:c r="AD13" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/145页眉下的图片被识别为表格一部分.docx--2aafe56f9445.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -1843,13 +1846,13 @@
         <x:v>0.9444</x:v>
       </x:c>
       <x:c r="AB14" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/168_3b1e2bb2ac/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/168删除线问题复现.pdf--3de2b5b29990.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC14" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/168_3b1e2bb2ac.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/168删除线问题复现.pdf.json</x:v>
       </x:c>
       <x:c r="AD14" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/168删除线问题复现.pdf--3de2b5b29990.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -1919,13 +1922,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB15" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/173_25a322df41/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/173图片中的公式未识别.pdf--7b41c1cff151.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC15" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/173_25a322df41.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/173图片中的公式未识别.pdf.json</x:v>
       </x:c>
       <x:c r="AD15" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/173图片中的公式未识别.pdf--7b41c1cff151.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -1991,13 +1994,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB16" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/177_cc5649b6dd/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/177两行三列表问题手绘多个流程图.docx--8042e0990aff.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC16" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/177_cc5649b6dd.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/177两行三列表问题手绘多个流程图.docx.json</x:v>
       </x:c>
       <x:c r="AD16" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/177两行三列表问题手绘多个流程图.docx--8042e0990aff.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -2067,13 +2070,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB17" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/183LC-ZXQ1-FAB5_f836930dd3/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/183LC-ZXQ1 FAB5表格列错位.docx--599b5aee4c7a.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC17" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/183LC-ZXQ1-FAB5_f836930dd3.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/183LC-ZXQ1 FAB5表格列错位.docx.json</x:v>
       </x:c>
       <x:c r="AD17" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/183LC-ZXQ1 FAB5表格列错位.docx--599b5aee4c7a.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
@@ -2139,13 +2142,13 @@
         <x:v>0.5911</x:v>
       </x:c>
       <x:c r="AB18" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/197PPT_3a6b363482/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/197PPT中的截图被拆分.pptx--d234d5a8b12d.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC18" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/197PPT_3a6b363482.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/197PPT中的截图被拆分.pptx.json</x:v>
       </x:c>
       <x:c r="AD18" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/197PPT中的截图被拆分.pptx--d234d5a8b12d.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
@@ -2215,13 +2218,13 @@
         <x:v>0.8886</x:v>
       </x:c>
       <x:c r="AB19" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/199_5f6b65dbd2/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/199行合并单元格被拆分.docx--38fccc66a3bd.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC19" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/199_5f6b65dbd2.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/199行合并单元格被拆分.docx.json</x:v>
       </x:c>
       <x:c r="AD19" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/199行合并单元格被拆分.docx--38fccc66a3bd.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
@@ -2291,13 +2294,13 @@
         <x:v>0.9417</x:v>
       </x:c>
       <x:c r="AB20" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/199_1a9a8e399b/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/199行合并单元格被拆分.pdf--43300200764b.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC20" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/199_1a9a8e399b.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/199行合并单元格被拆分.pdf.json</x:v>
       </x:c>
       <x:c r="AD20" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/199行合并单元格被拆分.pdf--43300200764b.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -2363,13 +2366,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB21" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/213_06f657f15d/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/213流程图表被识别为一张图片.docx--3c38334071dd.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC21" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/213_06f657f15d.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/213流程图表被识别为一张图片.docx.json</x:v>
       </x:c>
       <x:c r="AD21" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/213流程图表被识别为一张图片.docx--3c38334071dd.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
@@ -2443,13 +2446,13 @@
         <x:v>0.9888</x:v>
       </x:c>
       <x:c r="AB22" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/22_80b4ec1c1b/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/22芯片技术，从硅晶到智能未来.pptx--a5473b5075b2.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC22" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/22_80b4ec1c1b.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/22芯片技术，从硅晶到智能未来.pptx.json</x:v>
       </x:c>
       <x:c r="AD22" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/22芯片技术，从硅晶到智能未来.pptx--a5473b5075b2.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -2515,13 +2518,13 @@
         <x:v>0.9142</x:v>
       </x:c>
       <x:c r="AB23" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/35_a133e063ce/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/35测试问题验证.pdf--4beb15adb319.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC23" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/35_a133e063ce.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/35测试问题验证.pdf.json</x:v>
       </x:c>
       <x:c r="AD23" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/35测试问题验证.pdf--4beb15adb319.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
@@ -2583,13 +2586,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB24" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/58_c9982e148f/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58测试表格变文本.docx--7bc0b79f67c4.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC24" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/58_c9982e148f.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/58测试表格变文本.docx.json</x:v>
       </x:c>
       <x:c r="AD24" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58测试表格变文本.docx--7bc0b79f67c4.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -2659,13 +2662,13 @@
         <x:v>0.8483</x:v>
       </x:c>
       <x:c r="AB25" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/58-_-_10-case_0a5b21bc9a/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58多线表_纯白无外框_10页更多case.pptx--c1179a4a375d.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC25" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/58-_-_10-case_0a5b21bc9a.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/58多线表_纯白无外框_10页更多case.pptx.json</x:v>
       </x:c>
       <x:c r="AD25" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58多线表_纯白无外框_10页更多case.pptx--c1179a4a375d.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
@@ -2727,13 +2730,13 @@
         <x:v>0.9197</x:v>
       </x:c>
       <x:c r="AB26" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/58_e6e56991d3/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58多线表上方的文字被识别为表格内内容.pdf--a449b57f3a4d.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC26" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/58_e6e56991d3.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/58多线表上方的文字被识别为表格内内容.pdf.json</x:v>
       </x:c>
       <x:c r="AD26" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58多线表上方的文字被识别为表格内内容.pdf--a449b57f3a4d.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
@@ -2803,13 +2806,13 @@
         <x:v>0.7209</x:v>
       </x:c>
       <x:c r="AB27" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/58_dd6e34332e/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58企业复杂绩效指标与深度战略分析.pdf--f27b6409f9e2.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC27" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/58_dd6e34332e.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/58企业复杂绩效指标与深度战略分析.pdf.json</x:v>
       </x:c>
       <x:c r="AD27" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/58企业复杂绩效指标与深度战略分析.pdf--f27b6409f9e2.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
@@ -2867,13 +2870,13 @@
         <x:v>0.825</x:v>
       </x:c>
       <x:c r="AB28" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/80_5a74ba3173/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/80表格多行被识别成多行单元格.docx--4d777006c3f0.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC28" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/80_5a74ba3173.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/80表格多行被识别成多行单元格.docx.json</x:v>
       </x:c>
       <x:c r="AD28" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/80表格多行被识别成多行单元格.docx--4d777006c3f0.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
@@ -2935,13 +2938,13 @@
         <x:v>0.9339</x:v>
       </x:c>
       <x:c r="AB29" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/82_4c6010a653/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/82多行公式单页特殊情况构建.pptx--c6194a517e06.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC29" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/82_4c6010a653.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/82多行公式单页特殊情况构建.pptx.json</x:v>
       </x:c>
       <x:c r="AD29" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/82多行公式单页特殊情况构建.pptx--c6194a517e06.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -3011,13 +3014,13 @@
         <x:v>0.9708</x:v>
       </x:c>
       <x:c r="AB30" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/82-2_f8a05ad658/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/82公式识别线性回归 2.pptx--1c25b542c56c.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC30" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/82-2_f8a05ad658.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/82公式识别线性回归 2.pptx.json</x:v>
       </x:c>
       <x:c r="AD30" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/82公式识别线性回归 2.pptx--1c25b542c56c.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
@@ -3083,13 +3086,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB31" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/83_9a8a0ef637/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/83文字识别错误.docx--4e37b266b997.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC31" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/83_9a8a0ef637.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/83文字识别错误.docx.json</x:v>
       </x:c>
       <x:c r="AD31" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/83文字识别错误.docx--4e37b266b997.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
@@ -3151,13 +3154,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB32" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/84-12_faed7c59a2/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/84&amp;12合并单元格被拆分异常情况.docx--7e93e5ce7ad7.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC32" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/84-12_faed7c59a2.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/84&amp;12合并单元格被拆分异常情况.docx.json</x:v>
       </x:c>
       <x:c r="AD32" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/84&amp;12合并单元格被拆分异常情况.docx--7e93e5ce7ad7.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
@@ -3235,13 +3238,13 @@
         <x:v>0.9828</x:v>
       </x:c>
       <x:c r="AB33" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/86-YMS_mock_page14_fd122c7dee/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/86版式识别和公式YMS_mock_page14.pptx--409c2dbff424.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC33" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/86-YMS_mock_page14_fd122c7dee.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/86版式识别和公式YMS_mock_page14.pptx.json</x:v>
       </x:c>
       <x:c r="AD33" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/86版式识别和公式YMS_mock_page14.pptx--409c2dbff424.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
@@ -3299,13 +3302,13 @@
         <x:v>0.915</x:v>
       </x:c>
       <x:c r="AB34" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/86PPT-9_2f0b0d8ef7/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/86PPT板式识别不好9台.pptx--6f69d164879d.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC34" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/86PPT-9_2f0b0d8ef7.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/86PPT板式识别不好9台.pptx.json</x:v>
       </x:c>
       <x:c r="AD34" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/86PPT板式识别不好9台.pptx--6f69d164879d.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
@@ -3375,13 +3378,13 @@
         <x:v>0.8269</x:v>
       </x:c>
       <x:c r="AB35" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/97TagDes_1251b61763/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/97TagDes带正文识别为标题.pdf--5d0ade90f390.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC35" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/97TagDes_1251b61763.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/97TagDes带正文识别为标题.pdf.json</x:v>
       </x:c>
       <x:c r="AD35" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/97TagDes带正文识别为标题.pdf--5d0ade90f390.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
@@ -3451,13 +3454,13 @@
         <x:v>0.94</x:v>
       </x:c>
       <x:c r="AB36" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/98-3000_775000eed7/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/98 3000页页眉页脚误识别为标题.docx--41bb2d08b54b.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC36" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/98-3000_775000eed7.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/98 3000页页眉页脚误识别为标题.docx.json</x:v>
       </x:c>
       <x:c r="AD36" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/98 3000页页眉页脚误识别为标题.docx--41bb2d08b54b.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
@@ -3523,13 +3526,13 @@
         <x:v>0.713</x:v>
       </x:c>
       <x:c r="AB37" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/_01_6b76bc058a/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/基础解析_01.pdf--c5eec9324671.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC37" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/_01_6b76bc058a.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/基础解析_01.pdf.json</x:v>
       </x:c>
       <x:c r="AD37" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/基础解析_01.pdf--c5eec9324671.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
@@ -3603,13 +3606,13 @@
         <x:v>0.91</x:v>
       </x:c>
       <x:c r="AB38" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/__2a42f56ac6/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/中芯国际文档解析项目_鱼骨图.pdf--84949e249544.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC38" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/__2a42f56ac6.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/中芯国际文档解析项目_鱼骨图.pdf.json</x:v>
       </x:c>
       <x:c r="AD38" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/中芯国际文档解析项目_鱼骨图.pdf--84949e249544.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
@@ -3642,10 +3645,10 @@
         <x:v>0.7243</x:v>
       </x:c>
       <x:c r="M39" s="22" t="n">
-        <x:v>0.824</x:v>
+        <x:v>0.863</x:v>
       </x:c>
       <x:c r="N39" s="22" t="n">
-        <x:v>0.9302</x:v>
+        <x:v>0.9524</x:v>
       </x:c>
       <x:c r="O39" s="16"/>
       <x:c r="P39" s="16"/>
@@ -3673,23 +3676,23 @@
       </x:c>
       <x:c r="Y39" s="22" t="n">
         <x:f>AVERAGE(E39:N39)</x:f>
-        <x:v>0.8924142857142857</x:v>
+        <x:v>0.9011571428571429</x:v>
       </x:c>
       <x:c r="Z39" s="22" t="n">
         <x:f>SUMPRODUCT(E39:N39,O39:X39)/SUM(O39:X39)</x:f>
-        <x:v>0.9349241758241758</x:v>
+        <x:v>0.9470890109890111</x:v>
       </x:c>
       <x:c r="AA39" s="22" t="n">
-        <x:v>0.9349</x:v>
+        <x:v>0.9471</x:v>
       </x:c>
       <x:c r="AB39" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/08_5dea22a917/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页眉下的图片被识别为表格的一部分.doc--e4e8ed278023.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC39" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/08_5dea22a917.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/08页眉下的图片被识别为表格的一部分.doc.json</x:v>
       </x:c>
       <x:c r="AD39" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/08页眉下的图片被识别为表格的一部分.doc--e4e8ed278023.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
@@ -3709,20 +3712,20 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H40" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I40" s="22" t="n">
-        <x:v>0.981</x:v>
+        <x:v>0.864</x:v>
       </x:c>
       <x:c r="J40" s="22"/>
       <x:c r="K40" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.745</x:v>
       </x:c>
       <x:c r="L40" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7297</x:v>
       </x:c>
       <x:c r="M40" s="22" t="n">
-        <x:v>0.8256</x:v>
+        <x:v>0.8391</x:v>
       </x:c>
       <x:c r="N40" s="22" t="n">
         <x:v>0.8421</x:v>
@@ -3753,23 +3756,23 @@
       </x:c>
       <x:c r="Y40" s="22" t="n">
         <x:f>AVERAGE(E40:N40)</x:f>
-        <x:v>0.9498142857142857</x:v>
+        <x:v>0.7171285714285716</x:v>
       </x:c>
       <x:c r="Z40" s="22" t="n">
         <x:f>SUMPRODUCT(E40:N40,O40:X40)/SUM(O40:X40)</x:f>
-        <x:v>0.9239830985915494</x:v>
+        <x:v>0.7939366197183099</x:v>
       </x:c>
       <x:c r="AA40" s="22" t="n">
-        <x:v>0.924</x:v>
+        <x:v>0.7939</x:v>
       </x:c>
       <x:c r="AB40" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/35-V2_af5579a205/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/35表格内图片偏差V2.doc--f90fe3387072.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC40" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/35-V2_af5579a205.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/35表格内图片偏差V2.doc.json</x:v>
       </x:c>
       <x:c r="AD40" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/35表格内图片偏差V2.doc--f90fe3387072.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
@@ -3794,10 +3797,10 @@
       </x:c>
       <x:c r="J41" s="22"/>
       <x:c r="K41" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9991</x:v>
       </x:c>
       <x:c r="L41" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9444</x:v>
       </x:c>
       <x:c r="M41" s="22" t="n">
         <x:v>0.6639</x:v>
@@ -3825,23 +3828,23 @@
       <x:c r="X41" s="16"/>
       <x:c r="Y41" s="22" t="n">
         <x:f>AVERAGE(E41:N41)</x:f>
-        <x:v>0.9327799999999999</x:v>
+        <x:v>0.9214800000000001</x:v>
       </x:c>
       <x:c r="Z41" s="22" t="n">
         <x:f>SUMPRODUCT(E41:N41,O41:X41)/SUM(O41:X41)</x:f>
-        <x:v>0.8879666666666667</x:v>
+        <x:v>0.8832583333333334</x:v>
       </x:c>
       <x:c r="AA41" s="22" t="n">
-        <x:v>0.888</x:v>
+        <x:v>0.8833</x:v>
       </x:c>
       <x:c r="AB41" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/80_9462d3edae/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/80复杂表格空行保留.doc--7127914cba79.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC41" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/80_9462d3edae.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/80复杂表格空行保留.doc.json</x:v>
       </x:c>
       <x:c r="AD41" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/80复杂表格空行保留.doc--7127914cba79.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
@@ -3915,13 +3918,13 @@
         <x:v>0.9957</x:v>
       </x:c>
       <x:c r="AB42" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/135_515a221b44/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/135标题未识别.docx--9e9df3521855.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC42" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/135_515a221b44.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/135标题未识别.docx.json</x:v>
       </x:c>
       <x:c r="AD42" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/135标题未识别.docx--9e9df3521855.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
@@ -3991,13 +3994,13 @@
         <x:v>0.9809</x:v>
       </x:c>
       <x:c r="AB43" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/138_11abc15a4e/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/138参考文件标题格式丢失.pdf--3baf43dc55cb.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC43" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/138_11abc15a4e.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/138参考文件标题格式丢失.pdf.json</x:v>
       </x:c>
       <x:c r="AD43" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/138参考文件标题格式丢失.pdf--3baf43dc55cb.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
@@ -4071,13 +4074,13 @@
         <x:v>0.9993</x:v>
       </x:c>
       <x:c r="AB44" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/15unmerge_e872a58a8c/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/15unmerge合并单元格.docx--e0947abdee8c.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC44" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/15unmerge_e872a58a8c.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/15unmerge合并单元格.docx.json</x:v>
       </x:c>
       <x:c r="AD44" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/15unmerge合并单元格.docx--e0947abdee8c.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
@@ -4143,13 +4146,13 @@
         <x:v>0.9762</x:v>
       </x:c>
       <x:c r="AB45" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/162_e72dc3ea59/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/162块级公式数错误.pptx--0a5e2a427079.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC45" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/162_e72dc3ea59.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/162块级公式数错误.pptx.json</x:v>
       </x:c>
       <x:c r="AD45" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/162块级公式数错误.pptx--0a5e2a427079.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
@@ -4215,13 +4218,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AB46" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/165_c1a8b04492/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/165流程图表格中流程图识别为文字.docx--3f2bdb9c73a5.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC46" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/165_c1a8b04492.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/165流程图表格中流程图识别为文字.docx.json</x:v>
       </x:c>
       <x:c r="AD46" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/165流程图表格中流程图识别为文字.docx--3f2bdb9c73a5.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
@@ -4287,13 +4290,13 @@
         <x:v>0.7003</x:v>
       </x:c>
       <x:c r="AB47" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/180_f986199761/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/180标题和页眉相似丢失标题.doc--2f2741f38278.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC47" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/180_f986199761.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/180标题和页眉相似丢失标题.doc.json</x:v>
       </x:c>
       <x:c r="AD47" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/180标题和页眉相似丢失标题.doc--2f2741f38278.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
@@ -4367,13 +4370,13 @@
         <x:v>0.9935</x:v>
       </x:c>
       <x:c r="AB48" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/QR_a68e360e86/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/跨页表合并QR.pdf--131b5120bd7e.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC48" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/QR_a68e360e86.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/跨页表合并QR.pdf.json</x:v>
       </x:c>
       <x:c r="AD48" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/跨页表合并QR.pdf--131b5120bd7e.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
@@ -4443,13 +4446,13 @@
         <x:v>0.7409</x:v>
       </x:c>
       <x:c r="AB49" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/97TagDes_3770cb523c/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/97TagDes带正文识别为标题.docx--65e17ed6aaa4.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC49" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/97TagDes_3770cb523c.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/97TagDes带正文识别为标题.docx.json</x:v>
       </x:c>
       <x:c r="AD49" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/97TagDes带正文识别为标题.docx--65e17ed6aaa4.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
@@ -4523,13 +4526,13 @@
         <x:v>0.8898</x:v>
       </x:c>
       <x:c r="AB50" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/APFP-Description-Document1_4a2fab45d9/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/APFP Description Document1-已融合.pdf--9dffe40361c3.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC50" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/APFP-Description-Document1_4a2fab45d9.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/APFP Description Document1-已融合.pdf.json</x:v>
       </x:c>
       <x:c r="AD50" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/APFP Description Document1-已融合.pdf--9dffe40361c3.zip</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
@@ -4587,19 +4590,19 @@
         <x:v>0.4178</x:v>
       </x:c>
       <x:c r="AB51" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/cases/93_6b36bd45dc/parses/idc-4.1.14/parse.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/93大的流程图别切成多个小图片.pdf--a074b020027c.zip::_parse.json</x:v>
       </x:c>
       <x:c r="AC51" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/goldens/93_6b36bd45dc.json</x:v>
+        <x:v>datasets/半导体场景模拟数据golden/93大的流程图别切成多个小图片.pdf.json</x:v>
       </x:c>
       <x:c r="AD51" s="5" t="str">
-        <x:v>/Users/wangyaqi/Documents/cursor_project/moi-parse-bench/datasets/parse/evaluation-runs/eval_20260731_034612_dbc092/run.json</x:v>
+        <x:v>runs/半导体场景私有数据集-idc-4.1.14/93大的流程图别切成多个小图片.pdf--a074b020027c.zip</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab9442e08faa46f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f84f7f73ed246c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16150,19 +16153,19 @@
         <x:v>text_content</x:v>
       </x:c>
       <x:c r="E380" s="22" t="n">
-        <x:v>0.8589</x:v>
+        <x:v>0.8638</x:v>
       </x:c>
       <x:c r="F380" s="22" t="n">
-        <x:v>0.7918</x:v>
+        <x:v>0.8621</x:v>
       </x:c>
       <x:c r="G380" s="22" t="n">
-        <x:v>0.824</x:v>
+        <x:v>0.863</x:v>
       </x:c>
       <x:c r="H380" s="16" t="n">
         <x:v>17</x:v>
       </x:c>
       <x:c r="I380" s="16" t="n">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="J380" s="24" t="b">
         <x:v>0</x:v>
@@ -16184,19 +16187,19 @@
         <x:v>title_hierarchy</x:v>
       </x:c>
       <x:c r="E381" s="22" t="n">
-        <x:v>0.8696</x:v>
+        <x:v>0.9091</x:v>
       </x:c>
       <x:c r="F381" s="22" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="G381" s="22" t="n">
-        <x:v>0.9302</x:v>
+        <x:v>0.9524</x:v>
       </x:c>
       <x:c r="H381" s="16" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="I381" s="16" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J381" s="24" t="b">
         <x:v>0</x:v>
@@ -16304,19 +16307,19 @@
         <x:v>image</x:v>
       </x:c>
       <x:c r="E385" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F385" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G385" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H385" s="16" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="I385" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J385" s="24" t="b">
         <x:v>0</x:v>
@@ -16338,13 +16341,13 @@
         <x:v>layout</x:v>
       </x:c>
       <x:c r="E386" s="22" t="n">
-        <x:v>0.9874</x:v>
+        <x:v>0.9118</x:v>
       </x:c>
       <x:c r="F386" s="22" t="n">
-        <x:v>0.9706</x:v>
+        <x:v>0.7941</x:v>
       </x:c>
       <x:c r="G386" s="22" t="n">
-        <x:v>0.981</x:v>
+        <x:v>0.864</x:v>
       </x:c>
       <x:c r="H386" s="16" t="n">
         <x:v>34</x:v>
@@ -16398,24 +16401,26 @@
         <x:v>table</x:v>
       </x:c>
       <x:c r="E388" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.745</x:v>
       </x:c>
       <x:c r="F388" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.745</x:v>
       </x:c>
       <x:c r="G388" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.745</x:v>
       </x:c>
       <x:c r="H388" s="16" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I388" s="16" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J388" s="24" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="K388" s="16"/>
+      <x:c r="K388" s="16" t="str">
+        <x:v>contract_missing:table_embedded_images:embedded_block_uuids empty &amp; no image.contained_in &amp; table_html has no image markers</x:v>
+      </x:c>
       <x:c r="L388" s="16"/>
     </x:row>
     <x:row r="389" ht="15" hidden="0" customHeight="1">
@@ -16432,13 +16437,13 @@
         <x:v>table_teds</x:v>
       </x:c>
       <x:c r="E389" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7297</x:v>
       </x:c>
       <x:c r="F389" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7297</x:v>
       </x:c>
       <x:c r="G389" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.7297</x:v>
       </x:c>
       <x:c r="H389" s="16" t="n">
         <x:v>1</x:v>
@@ -16466,13 +16471,13 @@
         <x:v>text_content</x:v>
       </x:c>
       <x:c r="E390" s="22" t="n">
-        <x:v>0.95</x:v>
+        <x:v>0.9688</x:v>
       </x:c>
       <x:c r="F390" s="22" t="n">
-        <x:v>0.73</x:v>
+        <x:v>0.74</x:v>
       </x:c>
       <x:c r="G390" s="22" t="n">
-        <x:v>0.8256</x:v>
+        <x:v>0.8391</x:v>
       </x:c>
       <x:c r="H390" s="16" t="n">
         <x:v>20</x:v>
@@ -16706,13 +16711,13 @@
         <x:v>table</x:v>
       </x:c>
       <x:c r="E398" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9991</x:v>
       </x:c>
       <x:c r="F398" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9991</x:v>
       </x:c>
       <x:c r="G398" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9991</x:v>
       </x:c>
       <x:c r="H398" s="16" t="n">
         <x:v>2</x:v>
@@ -16740,13 +16745,13 @@
         <x:v>table_teds</x:v>
       </x:c>
       <x:c r="E399" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9444</x:v>
       </x:c>
       <x:c r="F399" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9444</x:v>
       </x:c>
       <x:c r="G399" s="22" t="n">
-        <x:v>1</x:v>
+        <x:v>0.9444</x:v>
       </x:c>
       <x:c r="H399" s="16" t="n">
         <x:v>2</x:v>
@@ -19887,7 +19892,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra734e4e610df4126"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a5aef826ea54cc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>